<commit_message>
Refactor product identifier in importation components to use productCode instead of barcode.
</commit_message>
<xml_diff>
--- a/public/templates/importationTemplate.xlsx
+++ b/public/templates/importationTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronal\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9145A40-C317-4DA0-9370-069F84BAB789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A84EF12-9BFC-404F-9E0D-23024D17A359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A22FCB21-30C0-4F19-B214-CE7F03932F0C}"/>
+    <workbookView xWindow="1728" yWindow="2208" windowWidth="17280" windowHeight="8880" xr2:uid="{A22FCB21-30C0-4F19-B214-CE7F03932F0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,13 +37,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>barcode</t>
-  </si>
-  <si>
     <t>quantity</t>
   </si>
   <si>
     <t>unitCost</t>
+  </si>
+  <si>
+    <t>productCode</t>
   </si>
 </sst>
 </file>
@@ -409,15 +409,15 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>